<commit_message>
Move Returns Summary/Detail/Unit Histories to after TEMU in the Sales Report
Sheet order is now: Summary, AMAZON, BM, EBAY, ONBUY, TEMU, Returns
Summary, Returns Detail, Unit Histories — per-channel sale detail reads
first, the returns lifecycle follows. Re-verified with 4 E2E suites
(the new return-restore scenario, the broader Inventory+Sales Report
round-trip against templates/samples, the Temu marketplace flow, and
the full upload → process-return flow) — 88/88 checks passing, template
fixtures round-trip cleanly through the new sheet layout.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/temu-marketplace/downloaded-sales-report.xlsx
+++ b/e2e-screenshots/temu-marketplace/downloaded-sales-report.xlsx
@@ -5,19 +5,21 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Summary" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Returns" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="AMAZON" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="BM" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="EBAY" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="ONBUY" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="TEMU" state="visible" r:id="rId10"/>
+    <sheet sheetId="2" name="AMAZON" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="BM" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="EBAY" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="ONBUY" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="TEMU" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="Returns Summary" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Returns Detail" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Unit Histories" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="95">
   <si>
     <t>Sales Report — Audit Summary</t>
   </si>
@@ -94,24 +96,75 @@
     <t>• Per-marketplace sheets carry a TOTAL row at the bottom summing every row shown there (active + returned) via SUM formulas — the Returns tab breaks the returned rows out on their own.</t>
   </si>
   <si>
-    <t>Sale Date</t>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Order Number</t>
+  </si>
+  <si>
+    <t>SKU</t>
+  </si>
+  <si>
+    <t>IMEI</t>
+  </si>
+  <si>
+    <t>Supplier</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>BP</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>SP-BP</t>
+  </si>
+  <si>
+    <t>Marginal Tax</t>
+  </si>
+  <si>
+    <t>Commission</t>
+  </si>
+  <si>
+    <t>C. VAT</t>
+  </si>
+  <si>
+    <t>DSF</t>
+  </si>
+  <si>
+    <t>DSF. VAT</t>
+  </si>
+  <si>
+    <t>Postage</t>
+  </si>
+  <si>
+    <t>P. VAT</t>
+  </si>
+  <si>
+    <t>Accessories</t>
+  </si>
+  <si>
+    <t>Total VAT</t>
+  </si>
+  <si>
+    <t>GP</t>
+  </si>
+  <si>
+    <t>GP %</t>
+  </si>
+  <si>
+    <t>Total VAT NTP</t>
+  </si>
+  <si>
+    <t>Comments</t>
   </si>
   <si>
     <t>Return Date</t>
   </si>
   <si>
-    <t>Order Number</t>
-  </si>
-  <si>
-    <t>SKU</t>
-  </si>
-  <si>
-    <t>IMEI</t>
-  </si>
-  <si>
-    <t>Supplier</t>
-  </si>
-  <si>
     <t>Outcome</t>
   </si>
   <si>
@@ -121,63 +174,6 @@
     <t>Shipping Legs</t>
   </si>
   <si>
-    <t>BP</t>
-  </si>
-  <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>SP-BP</t>
-  </si>
-  <si>
-    <t>Postage</t>
-  </si>
-  <si>
-    <t>Comments</t>
-  </si>
-  <si>
-    <t>No returns recorded for this period.</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Quantity</t>
-  </si>
-  <si>
-    <t>Marginal Tax</t>
-  </si>
-  <si>
-    <t>Commission</t>
-  </si>
-  <si>
-    <t>C. VAT</t>
-  </si>
-  <si>
-    <t>DSF</t>
-  </si>
-  <si>
-    <t>DSF. VAT</t>
-  </si>
-  <si>
-    <t>P. VAT</t>
-  </si>
-  <si>
-    <t>Accessories</t>
-  </si>
-  <si>
-    <t>Total VAT</t>
-  </si>
-  <si>
-    <t>GP</t>
-  </si>
-  <si>
-    <t>GP %</t>
-  </si>
-  <si>
-    <t>Total VAT NTP</t>
-  </si>
-  <si>
     <t>Postage Loss</t>
   </si>
   <si>
@@ -221,6 +217,93 @@
   </si>
   <si>
     <t>MHL</t>
+  </si>
+  <si>
+    <t>Period</t>
+  </si>
+  <si>
+    <t>All Time</t>
+  </si>
+  <si>
+    <t>Total Returns</t>
+  </si>
+  <si>
+    <t>Total Postage Loss £</t>
+  </si>
+  <si>
+    <t>Avg Loss per Return £</t>
+  </si>
+  <si>
+    <t>Carriage cost policy</t>
+  </si>
+  <si>
+    <t>Refund / Repair / To-Supplier</t>
+  </si>
+  <si>
+    <t>2 legs (outbound + inbound)</t>
+  </si>
+  <si>
+    <t>Replacement</t>
+  </si>
+  <si>
+    <t>3 legs (+ replacement outbound)</t>
+  </si>
+  <si>
+    <t>Leg cost</t>
+  </si>
+  <si>
+    <t>postage + P.VAT, snapshotted at return time</t>
+  </si>
+  <si>
+    <t>Pre-tracking cutoff</t>
+  </si>
+  <si>
+    <t>Carriage costed from</t>
+  </si>
+  <si>
+    <t>no costed returns in this period</t>
+  </si>
+  <si>
+    <t>Uncosted (pre-tracking) returns</t>
+  </si>
+  <si>
+    <t>Unit IMEI</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>Storage</t>
+  </si>
+  <si>
+    <t>Colour</t>
+  </si>
+  <si>
+    <t>Original Sale Date</t>
+  </si>
+  <si>
+    <t>Original Sale Price</t>
+  </si>
+  <si>
+    <t>Return Type</t>
+  </si>
+  <si>
+    <t>Reason</t>
+  </si>
+  <si>
+    <t>Leg Cost £</t>
+  </si>
+  <si>
+    <t>Event Date</t>
+  </si>
+  <si>
+    <t>Event</t>
+  </si>
+  <si>
+    <t>Detail</t>
+  </si>
+  <si>
+    <t>Amount £</t>
   </si>
 </sst>
 </file>
@@ -230,7 +313,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yyyy"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -244,10 +327,6 @@
     </font>
     <font>
       <b/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF64748B"/>
     </font>
   </fonts>
   <fills count="4">
@@ -280,7 +359,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -288,7 +367,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -921,75 +999,93 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="11" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="17" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="30" customWidth="1"/>
-    <col min="11" max="11" width="13" customWidth="1"/>
-    <col min="12" max="13" width="8" customWidth="1"/>
-    <col min="16" max="16" width="24" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="C1" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="D1" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="E1" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="F1" t="s">
         <v>30</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="G1" t="s">
         <v>31</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="H1" t="s">
         <v>32</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="I1" t="s">
         <v>33</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="2" t="s">
+      <c r="J1" t="s">
         <v>34</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="K1" t="s">
         <v>35</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="L1" t="s">
         <v>36</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="M1" t="s">
         <v>37</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="N1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="O1" t="s">
         <v>39</v>
+      </c>
+      <c r="P1" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>41</v>
+      </c>
+      <c r="R1" t="s">
+        <v>42</v>
+      </c>
+      <c r="S1" t="s">
+        <v>43</v>
+      </c>
+      <c r="T1" t="s">
+        <v>44</v>
+      </c>
+      <c r="U1" t="s">
+        <v>45</v>
+      </c>
+      <c r="V1" t="s">
+        <v>46</v>
+      </c>
+      <c r="W1" t="s">
+        <v>47</v>
+      </c>
+      <c r="X1" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>49</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>51</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1000,92 +1096,83 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I1" t="s">
+        <v>33</v>
+      </c>
+      <c r="J1" t="s">
+        <v>34</v>
+      </c>
+      <c r="K1" t="s">
+        <v>35</v>
+      </c>
+      <c r="L1" t="s">
+        <v>52</v>
+      </c>
+      <c r="M1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="O1" t="s">
         <v>41</v>
       </c>
-      <c r="G1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H1" t="s">
-        <v>35</v>
-      </c>
-      <c r="I1" t="s">
-        <v>36</v>
-      </c>
-      <c r="J1" t="s">
-        <v>42</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="P1" t="s">
         <v>43</v>
       </c>
-      <c r="L1" t="s">
+      <c r="Q1" t="s">
         <v>44</v>
       </c>
-      <c r="M1" t="s">
+      <c r="R1" t="s">
         <v>45</v>
       </c>
-      <c r="N1" t="s">
+      <c r="S1" t="s">
         <v>46</v>
       </c>
-      <c r="O1" t="s">
-        <v>37</v>
-      </c>
-      <c r="P1" t="s">
+      <c r="T1" t="s">
         <v>47</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="U1" t="s">
         <v>48</v>
       </c>
-      <c r="R1" t="s">
+      <c r="V1" t="s">
         <v>49</v>
       </c>
-      <c r="S1" t="s">
+      <c r="W1" t="s">
         <v>50</v>
       </c>
-      <c r="T1" t="s">
+      <c r="X1" t="s">
         <v>51</v>
       </c>
-      <c r="U1" t="s">
-        <v>52</v>
-      </c>
-      <c r="V1" t="s">
-        <v>38</v>
-      </c>
-      <c r="W1" t="s">
-        <v>26</v>
-      </c>
-      <c r="X1" t="s">
-        <v>31</v>
-      </c>
       <c r="Y1" t="s">
-        <v>32</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1097,83 +1184,101 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y1"/>
+  <dimension ref="A1:AE1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
         <v>27</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>28</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>29</v>
       </c>
-      <c r="E1" t="s">
-        <v>30</v>
-      </c>
       <c r="F1" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="G1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I1" t="s">
+        <v>33</v>
+      </c>
+      <c r="J1" t="s">
         <v>34</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>35</v>
-      </c>
-      <c r="I1" t="s">
-        <v>36</v>
-      </c>
-      <c r="J1" t="s">
-        <v>42</v>
-      </c>
-      <c r="K1" t="s">
-        <v>43</v>
       </c>
       <c r="L1" t="s">
         <v>54</v>
       </c>
       <c r="M1" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="N1" t="s">
+        <v>56</v>
+      </c>
+      <c r="O1" t="s">
+        <v>57</v>
+      </c>
+      <c r="P1" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>40</v>
+      </c>
+      <c r="R1" t="s">
+        <v>58</v>
+      </c>
+      <c r="S1" t="s">
+        <v>59</v>
+      </c>
+      <c r="T1" t="s">
+        <v>41</v>
+      </c>
+      <c r="U1" t="s">
+        <v>42</v>
+      </c>
+      <c r="V1" t="s">
+        <v>43</v>
+      </c>
+      <c r="W1" t="s">
+        <v>44</v>
+      </c>
+      <c r="X1" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Z1" t="s">
         <v>47</v>
       </c>
-      <c r="O1" t="s">
+      <c r="AA1" t="s">
         <v>48</v>
       </c>
-      <c r="P1" t="s">
+      <c r="AB1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AC1" t="s">
         <v>50</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="AD1" t="s">
         <v>51</v>
       </c>
-      <c r="R1" t="s">
-        <v>52</v>
-      </c>
-      <c r="S1" t="s">
-        <v>38</v>
-      </c>
-      <c r="T1" t="s">
-        <v>26</v>
-      </c>
-      <c r="U1" t="s">
-        <v>31</v>
-      </c>
-      <c r="V1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W1" t="s">
-        <v>33</v>
-      </c>
-      <c r="X1" t="s">
-        <v>53</v>
-      </c>
-      <c r="Y1" t="s">
+      <c r="AE1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1185,101 +1290,83 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K1" t="s">
+        <v>60</v>
+      </c>
+      <c r="L1" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" t="s">
-        <v>55</v>
-      </c>
-      <c r="G1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H1" t="s">
-        <v>35</v>
-      </c>
-      <c r="I1" t="s">
-        <v>36</v>
-      </c>
-      <c r="J1" t="s">
+      <c r="N1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O1" t="s">
         <v>42</v>
       </c>
-      <c r="K1" t="s">
+      <c r="P1" t="s">
         <v>43</v>
       </c>
-      <c r="L1" t="s">
-        <v>56</v>
-      </c>
-      <c r="M1" t="s">
-        <v>57</v>
-      </c>
-      <c r="N1" t="s">
-        <v>58</v>
-      </c>
-      <c r="O1" t="s">
-        <v>59</v>
-      </c>
-      <c r="P1" t="s">
-        <v>37</v>
-      </c>
       <c r="Q1" t="s">
+        <v>44</v>
+      </c>
+      <c r="R1" t="s">
+        <v>45</v>
+      </c>
+      <c r="S1" t="s">
+        <v>46</v>
+      </c>
+      <c r="T1" t="s">
         <v>47</v>
       </c>
-      <c r="R1" t="s">
-        <v>60</v>
-      </c>
-      <c r="S1" t="s">
-        <v>61</v>
-      </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>48</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>49</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>50</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>51</v>
       </c>
-      <c r="X1" t="s">
-        <v>52</v>
-      </c>
       <c r="Y1" t="s">
-        <v>38</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>32</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1291,84 +1378,214 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y1"/>
+  <dimension ref="A1:Z3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I1" t="s">
+        <v>33</v>
+      </c>
+      <c r="J1" t="s">
+        <v>34</v>
+      </c>
+      <c r="K1" t="s">
+        <v>35</v>
+      </c>
+      <c r="L1" t="s">
+        <v>61</v>
+      </c>
+      <c r="M1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G1" t="s">
-        <v>35</v>
-      </c>
-      <c r="H1" t="s">
-        <v>36</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="O1" t="s">
+        <v>41</v>
+      </c>
+      <c r="P1" t="s">
         <v>42</v>
       </c>
-      <c r="J1" t="s">
+      <c r="Q1" t="s">
         <v>43</v>
       </c>
-      <c r="K1" t="s">
+      <c r="R1" t="s">
+        <v>44</v>
+      </c>
+      <c r="S1" t="s">
+        <v>45</v>
+      </c>
+      <c r="T1" t="s">
+        <v>46</v>
+      </c>
+      <c r="U1" t="s">
+        <v>47</v>
+      </c>
+      <c r="V1" t="s">
+        <v>48</v>
+      </c>
+      <c r="W1" t="s">
+        <v>49</v>
+      </c>
+      <c r="X1" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A2" s="7">
+        <v>46191.5</v>
+      </c>
+      <c r="B2" t="s">
         <v>62</v>
       </c>
-      <c r="L1" t="s">
-        <v>37</v>
-      </c>
-      <c r="M1" t="s">
-        <v>47</v>
-      </c>
-      <c r="N1" t="s">
-        <v>48</v>
-      </c>
-      <c r="O1" t="s">
-        <v>49</v>
-      </c>
-      <c r="P1" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>51</v>
-      </c>
-      <c r="R1" t="s">
-        <v>52</v>
-      </c>
-      <c r="S1" t="s">
-        <v>38</v>
-      </c>
-      <c r="T1" t="s">
-        <v>26</v>
-      </c>
-      <c r="U1" t="s">
-        <v>31</v>
-      </c>
-      <c r="V1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W1" t="s">
-        <v>33</v>
-      </c>
-      <c r="X1" t="s">
-        <v>53</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>10</v>
+      <c r="C2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" s="3">
+        <v>55</v>
+      </c>
+      <c r="H2" s="3">
+        <v>83.99</v>
+      </c>
+      <c r="I2" s="3">
+        <f>H2-G2</f>
+      </c>
+      <c r="J2" s="3">
+        <f>I2*16.67%</f>
+      </c>
+      <c r="K2" s="3">
+        <v>3.87</v>
+      </c>
+      <c r="L2" s="3">
+        <v>4.07</v>
+      </c>
+      <c r="M2" s="3">
+        <v>6.3</v>
+      </c>
+      <c r="N2" s="3">
+        <f>M2*20%</f>
+      </c>
+      <c r="O2" s="3">
+        <v>1</v>
+      </c>
+      <c r="P2" s="3">
+        <f>N2</f>
+      </c>
+      <c r="Q2" s="3">
+        <f>I2-J2-K2-M2-N2-O2</f>
+      </c>
+      <c r="R2" s="3">
+        <f>(Q2-Y2)/G2*100</f>
+      </c>
+      <c r="S2" s="3">
+        <f>J2-P2</f>
+      </c>
+      <c r="T2" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="3">
+        <f>Q2-Y2</f>
+      </c>
+    </row>
+    <row r="3" spans="1:26" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="9">
+        <f>SUM(F2:F2)</f>
+      </c>
+      <c r="G3" s="9">
+        <f>SUM(G2:G2)</f>
+      </c>
+      <c r="H3" s="9">
+        <f>SUM(H2:H2)</f>
+      </c>
+      <c r="I3" s="9">
+        <f>SUM(I2:I2)</f>
+      </c>
+      <c r="J3" s="9">
+        <f>SUM(J2:J2)</f>
+      </c>
+      <c r="K3" s="9">
+        <f>SUM(K2:K2)</f>
+      </c>
+      <c r="L3" s="9">
+        <f>SUM(L2:L2)</f>
+      </c>
+      <c r="M3" s="9">
+        <f>SUM(M2:M2)</f>
+      </c>
+      <c r="N3" s="9">
+        <f>SUM(N2:N2)</f>
+      </c>
+      <c r="O3" s="9">
+        <f>SUM(O2:O2)</f>
+      </c>
+      <c r="P3" s="9">
+        <f>SUM(P2:P2)</f>
+      </c>
+      <c r="Q3" s="9">
+        <f>SUM(Q2:Q2)</f>
+      </c>
+      <c r="R3" s="9">
+        <f>IFERROR((Q3-Y3)/G3*100,0)</f>
+      </c>
+      <c r="S3" s="9">
+        <f>SUM(S2:S2)</f>
+      </c>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="9">
+        <f>SUM(Y2:Y2)</f>
+      </c>
+      <c r="Z3" s="9">
+        <f>SUM(Z2:Z2)</f>
       </c>
     </row>
   </sheetData>
@@ -1379,214 +1596,218 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z3"/>
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B11" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>81</v>
+      </c>
+      <c r="B16">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:P1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="B1" t="s">
-        <v>27</v>
+        <v>82</v>
       </c>
       <c r="C1" t="s">
-        <v>28</v>
+        <v>83</v>
       </c>
       <c r="D1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1" t="s">
         <v>29</v>
       </c>
+      <c r="G1" t="s">
+        <v>86</v>
+      </c>
+      <c r="H1" t="s">
+        <v>87</v>
+      </c>
+      <c r="I1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J1" t="s">
+        <v>88</v>
+      </c>
+      <c r="K1" t="s">
+        <v>48</v>
+      </c>
+      <c r="L1" t="s">
+        <v>89</v>
+      </c>
+      <c r="M1" t="s">
+        <v>46</v>
+      </c>
+      <c r="N1" t="s">
+        <v>90</v>
+      </c>
+      <c r="O1" t="s">
+        <v>50</v>
+      </c>
+      <c r="P1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D1" t="s">
+        <v>92</v>
+      </c>
       <c r="E1" t="s">
-        <v>30</v>
+        <v>93</v>
       </c>
       <c r="F1" t="s">
-        <v>41</v>
+        <v>94</v>
       </c>
       <c r="G1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H1" t="s">
-        <v>35</v>
-      </c>
-      <c r="I1" t="s">
-        <v>36</v>
-      </c>
-      <c r="J1" t="s">
-        <v>42</v>
-      </c>
-      <c r="K1" t="s">
-        <v>43</v>
-      </c>
-      <c r="L1" t="s">
-        <v>63</v>
-      </c>
-      <c r="M1" t="s">
-        <v>37</v>
-      </c>
-      <c r="N1" t="s">
-        <v>47</v>
-      </c>
-      <c r="O1" t="s">
-        <v>48</v>
-      </c>
-      <c r="P1" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>50</v>
-      </c>
-      <c r="R1" t="s">
-        <v>51</v>
-      </c>
-      <c r="S1" t="s">
-        <v>52</v>
-      </c>
-      <c r="T1" t="s">
-        <v>38</v>
-      </c>
-      <c r="U1" t="s">
-        <v>26</v>
-      </c>
-      <c r="V1" t="s">
-        <v>31</v>
-      </c>
-      <c r="W1" t="s">
-        <v>32</v>
-      </c>
-      <c r="X1" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A2" s="8">
-        <v>46191.5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="E2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2" s="3">
-        <v>55</v>
-      </c>
-      <c r="H2" s="3">
-        <v>83.99</v>
-      </c>
-      <c r="I2" s="3">
-        <f>H2-G2</f>
-      </c>
-      <c r="J2" s="3">
-        <f>I2*16.67%</f>
-      </c>
-      <c r="K2" s="3">
-        <v>3.87</v>
-      </c>
-      <c r="L2" s="3">
-        <v>4.07</v>
-      </c>
-      <c r="M2" s="3">
-        <v>6.3</v>
-      </c>
-      <c r="N2" s="3">
-        <f>M2*20%</f>
-      </c>
-      <c r="O2" s="3">
-        <v>1</v>
-      </c>
-      <c r="P2" s="3">
-        <f>N2</f>
-      </c>
-      <c r="Q2" s="3">
-        <f>I2-J2-K2-M2-N2-O2</f>
-      </c>
-      <c r="R2" s="3">
-        <f>(Q2-Y2)/G2*100</f>
-      </c>
-      <c r="S2" s="3">
-        <f>J2-P2</f>
-      </c>
-      <c r="T2" t="s">
-        <v>1</v>
-      </c>
-      <c r="Z2" s="3">
-        <f>Q2-Y2</f>
-      </c>
-    </row>
-    <row r="3" spans="1:26" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="10">
-        <f>SUM(F2:F2)</f>
-      </c>
-      <c r="G3" s="10">
-        <f>SUM(G2:G2)</f>
-      </c>
-      <c r="H3" s="10">
-        <f>SUM(H2:H2)</f>
-      </c>
-      <c r="I3" s="10">
-        <f>SUM(I2:I2)</f>
-      </c>
-      <c r="J3" s="10">
-        <f>SUM(J2:J2)</f>
-      </c>
-      <c r="K3" s="10">
-        <f>SUM(K2:K2)</f>
-      </c>
-      <c r="L3" s="10">
-        <f>SUM(L2:L2)</f>
-      </c>
-      <c r="M3" s="10">
-        <f>SUM(M2:M2)</f>
-      </c>
-      <c r="N3" s="10">
-        <f>SUM(N2:N2)</f>
-      </c>
-      <c r="O3" s="10">
-        <f>SUM(O2:O2)</f>
-      </c>
-      <c r="P3" s="10">
-        <f>SUM(P2:P2)</f>
-      </c>
-      <c r="Q3" s="10">
-        <f>SUM(Q2:Q2)</f>
-      </c>
-      <c r="R3" s="10">
-        <f>IFERROR((Q3-Y3)/G3*100,0)</f>
-      </c>
-      <c r="S3" s="10">
-        <f>SUM(S2:S2)</f>
-      </c>
-      <c r="T3" s="6"/>
-      <c r="U3" s="6"/>
-      <c r="V3" s="6"/>
-      <c r="W3" s="6"/>
-      <c r="X3" s="6"/>
-      <c r="Y3" s="10">
-        <f>SUM(Y2:Y2)</f>
-      </c>
-      <c r="Z3" s="10">
-        <f>SUM(Z2:Z2)</f>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh final batch of E2E evidence — full historical sweep complete
All 28 reproducible E2E scripts in scripts/ re-run fresh against the
current codebase: 487/487 checks passing (including e2eBatchVsMarketplace
and e2eTemplateFillAndUpload, re-run individually with extra headroom
after hitting the sweep runner's 280s per-script cap mid-run, both
confirmed clean at 27/27 and 17/17).
</commit_message>
<xml_diff>
--- a/e2e-screenshots/temu-marketplace/downloaded-sales-report.xlsx
+++ b/e2e-screenshots/temu-marketplace/downloaded-sales-report.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="97">
   <si>
     <t>Sales Report — Audit Summary</t>
   </si>
@@ -294,6 +294,9 @@
     <t>Leg Cost £</t>
   </si>
   <si>
+    <t>No returns recorded for this period.</t>
+  </si>
+  <si>
     <t>Event Date</t>
   </si>
   <si>
@@ -304,6 +307,9 @@
   </si>
   <si>
     <t>Amount £</t>
+  </si>
+  <si>
+    <t>No unit return history to show for this period.</t>
   </si>
 </sst>
 </file>
@@ -313,7 +319,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yyyy"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -327,6 +333,10 @@
     </font>
     <font>
       <b/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF64748B"/>
     </font>
   </fonts>
   <fills count="4">
@@ -359,7 +369,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -370,6 +380,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1723,7 +1734,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -1774,6 +1785,11 @@
       </c>
       <c r="P1" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1784,7 +1800,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1795,19 +1811,24 @@
         <v>83</v>
       </c>
       <c r="C1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G1" t="s">
         <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>